<commit_message>
Strengthen tracking plan skill quality gates
</commit_message>
<xml_diff>
--- a/skill/assets/ga4_tracking_plan_template.xlsx
+++ b/skill/assets/ga4_tracking_plan_template.xlsx
@@ -317,7 +317,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -329,6 +329,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00EAF6F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3989,17 +3996,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Open the route and capture the rendered page state.</t>
+          <t>Skip or capture only with approved test access; do not use personal credentials.</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>capture_required</t>
+          <t>skip_allowed</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Capture during coverage or later QA when the journey is accessible.</t>
+          <t>Skip is allowed when approved credentials or a safe test environment are unavailable.</t>
         </is>
       </c>
     </row>
@@ -4017,18 +4024,21 @@
       <formula>"shared_evidence"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"skip_allowed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"capture_required"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"not_needed"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="G4:G209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"capture_required,captured,shared_evidence,not_needed,blocked"</formula1>
+      <formula1>"capture_required,captured,shared_evidence,skip_allowed,not_needed,blocked"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4435,10 +4445,10 @@
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
       <formula>"KO"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
       <formula>"Cannot test"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>